<commit_message>
test: expand phase 01 release readiness
</commit_message>
<xml_diff>
--- a/Back End/outputs/development-test-register/APS-Development-and-Test-Register-Phase-01.xlsx
+++ b/Back End/outputs/development-test-register/APS-Development-and-Test-Register-Phase-01.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra22ab517dc884de1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Register" sheetId="2" r:id="R66cf0bdda625407a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Log" sheetId="3" r:id="R7fe06a7ac7a34027"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="4" r:id="Rcd4b5e6cff7b4334"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Executions" sheetId="5" r:id="R975cbac192bd4cc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="6" r:id="Rcdb61b7f72c04982"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="7" r:id="R28046132485346ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R999a5b56e8494e5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Register" sheetId="2" r:id="R144d7cc2825e4c1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Log" sheetId="3" r:id="R2acb00e4f0374739"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="4" r:id="R4ac50ca2de2e48a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Executions" sheetId="5" r:id="Rc7d14a82ddf249d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="6" r:id="R794fe10da0c245ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="7" r:id="Ra2dbdc5c6fff40d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -44,7 +44,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -83,8 +83,18 @@
       <x:color rgb="FF15803D"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FFB91C1C"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF92400E"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -109,6 +119,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE8F5EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F5EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDECEC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4D6"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -154,7 +179,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="49">
+  <x:cellXfs count="57">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -272,6 +297,30 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -881,7 +930,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Refb06001ca164067"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R29995a806f344281"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1227,7 +1276,7 @@
         <x:v>Current</x:v>
       </x:c>
       <x:c r="D4" s="13" t="str">
-        <x:v>Phase 01 acceptance snapshot</x:v>
+        <x:v>Phase 01 release-readiness snapshot</x:v>
       </x:c>
       <x:c r="E4" s="36"/>
       <x:c r="F4" s="36"/>
@@ -1243,19 +1292,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D5" s="22" t="str">
-        <x:v>AG-P01-01</x:v>
+        <x:v>Functional suite</x:v>
       </x:c>
       <x:c r="E5" s="46" t="str">
-        <x:v>Identity persistence</x:v>
-      </x:c>
-      <x:c r="F5" s="22" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>27 passed</x:v>
+      </x:c>
+      <x:c r="F5" s="51" t="str">
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G5" s="22" t="str">
-        <x:v>Migrations and deterministic seed passed</x:v>
+        <x:v>90.59% coverage</x:v>
       </x:c>
       <x:c r="H5" s="22" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="60" hidden="0" customHeight="1">
@@ -1267,19 +1316,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>AG-P01-02</x:v>
+        <x:v>Database recovery</x:v>
       </x:c>
       <x:c r="E6" s="47" t="str">
-        <x:v>Authentication and sessions</x:v>
-      </x:c>
-      <x:c r="F6" s="23" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>Backup/restore</x:v>
+      </x:c>
+      <x:c r="F6" s="52" t="str">
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G6" s="23" t="str">
-        <x:v>Login, CSRF, expiry and revocation passed</x:v>
+        <x:v>Revision and sampled counts matched</x:v>
       </x:c>
       <x:c r="H6" s="23" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" hidden="0" customHeight="1">
@@ -1288,22 +1337,22 @@
       </x:c>
       <x:c r="B7" s="32" t="n">
         <x:f>COUNTIF('Test Executions'!$G$4:$G$60,"Passed")</x:f>
-        <x:v>42</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>AG-P01-03</x:v>
+        <x:v>Session resilience</x:v>
       </x:c>
       <x:c r="E7" s="47" t="str">
-        <x:v>RBAC boundaries</x:v>
-      </x:c>
-      <x:c r="F7" s="23" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>Concurrency/restart</x:v>
+      </x:c>
+      <x:c r="F7" s="52" t="str">
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G7" s="23" t="str">
-        <x:v>Role grants and explicit deny precedence passed</x:v>
+        <x:v>Distinct sessions; restart continuity</x:v>
       </x:c>
       <x:c r="H7" s="23" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="72" hidden="0" customHeight="1">
@@ -1312,22 +1361,22 @@
       </x:c>
       <x:c r="B8" s="32" t="n">
         <x:f>COUNTIF('Test Executions'!$G$4:$G$60,"Failed")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
-        <x:v>AG-P01-04</x:v>
+        <x:v>Python dependencies</x:v>
       </x:c>
       <x:c r="E8" s="47" t="str">
-        <x:v>Administration</x:v>
-      </x:c>
-      <x:c r="F8" s="23" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>pip-audit</x:v>
+      </x:c>
+      <x:c r="F8" s="54" t="str">
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
-        <x:v>CRUD, audit and manager association passed</x:v>
+        <x:v>Runtime vulnerabilities require remediation</x:v>
       </x:c>
       <x:c r="H8" s="23" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="60" hidden="0" customHeight="1">
@@ -1339,36 +1388,36 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>AG-P01-05</x:v>
+        <x:v>Frontend dependencies</x:v>
       </x:c>
       <x:c r="E9" s="47" t="str">
-        <x:v>Session hygiene</x:v>
-      </x:c>
-      <x:c r="F9" s="23" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>pnpm audit</x:v>
+      </x:c>
+      <x:c r="F9" s="54" t="str">
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
-        <x:v>Cleanup and production refusal passed</x:v>
+        <x:v>5 high and 4 moderate advisories</x:v>
       </x:c>
       <x:c r="H9" s="23" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" hidden="0" customHeight="1">
       <x:c r="D10" s="24" t="str">
-        <x:v>AG-P01-08</x:v>
+        <x:v>Browser matrix</x:v>
       </x:c>
       <x:c r="E10" s="48" t="str">
-        <x:v>Automated quality</x:v>
-      </x:c>
-      <x:c r="F10" s="24" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>Interactive/cross-browser</x:v>
+      </x:c>
+      <x:c r="F10" s="56" t="str">
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G10" s="24" t="str">
-        <x:v>23 tests; 90.46% coverage; build passed</x:v>
+        <x:v>Browser runtime and external browsers required</x:v>
       </x:c>
       <x:c r="H10" s="24" t="str">
-        <x:v>2026-08-26</x:v>
+        <x:v>2026-08-27</x:v>
       </x:c>
     </x:row>
     <x:row r="11"/>
@@ -1386,7 +1435,7 @@
       </x:c>
       <x:c r="E13" t="n">
         <x:f>B7</x:f>
-        <x:v>42</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -1395,7 +1444,7 @@
       </x:c>
       <x:c r="E14" t="n">
         <x:f>B8</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -1509,7 +1558,7 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="Pending"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc814d07e8c214121"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19d1701f29b14178"/>
 </x:worksheet>
 </file>
 
@@ -1622,7 +1671,7 @@
         <x:v>Backend Team</x:v>
       </x:c>
       <x:c r="I5" s="23" t="str">
-        <x:v>Commit a796a43; 23 tests passed; 90.46% coverage; frontend commit 7043f0f</x:v>
+        <x:v>27 tests passed; 90.59% coverage. Release blocked by dependency vulnerabilities and interactive browser validation gaps.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="120" hidden="0" customHeight="1">
@@ -1862,7 +1911,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a353bf6f2e54166"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb395cd659c0c43be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2980,7 +3029,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8edaab4e02584039"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3c87407b9124436"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4768,13 +4817,587 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="K45" s="41" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="L45" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M45" s="41" t="str">
+        <x:v>Implementation/build passed; actual downloaded workbook validation remains blocked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="60" customHeight="1">
+      <x:c r="A46" s="41" t="str">
+        <x:v>TC-P01-023</x:v>
+      </x:c>
+      <x:c r="B46" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C46" s="41" t="str">
+        <x:v>Dedicated test database lifecycle</x:v>
+      </x:c>
+      <x:c r="D46" s="41" t="str">
+        <x:v>Database</x:v>
+      </x:c>
+      <x:c r="E46" s="41" t="str">
+        <x:v>Empty payment_module_test database</x:v>
+      </x:c>
+      <x:c r="F46" s="41" t="str">
+        <x:v>Upgrade 0001-0004; seed twice; downgrade to base; replay to head</x:v>
+      </x:c>
+      <x:c r="G46" s="41" t="str">
+        <x:v>All migration and deterministic seed operations complete on the isolated database</x:v>
+      </x:c>
+      <x:c r="H46" s="41" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I46" s="41" t="str">
+        <x:v>alembic upgrade/downgrade/replay using TEST_DATABASE_URL</x:v>
+      </x:c>
+      <x:c r="J46" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K46" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L46" s="41" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="M45" s="41" t="str">
-        <x:v>XLSX export implementation and build passed</x:v>
+      <x:c r="M46" s="41" t="str">
+        <x:v>Isolated PostgreSQL 16 validation 2026-08-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="60" customHeight="1">
+      <x:c r="A47" s="41" t="str">
+        <x:v>TC-P01-024</x:v>
+      </x:c>
+      <x:c r="B47" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C47" s="41" t="str">
+        <x:v>Concurrent login and session fixation</x:v>
+      </x:c>
+      <x:c r="D47" s="41" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E47" s="41" t="str">
+        <x:v>Seeded administrator</x:v>
+      </x:c>
+      <x:c r="F47" s="41" t="str">
+        <x:v>Run four concurrent logins and supply an attacker-controlled cookie</x:v>
+      </x:c>
+      <x:c r="G47" s="41" t="str">
+        <x:v>Each login receives a distinct valid session; supplied cookie is replaced; HttpOnly/SameSite/Path flags are present</x:v>
+      </x:c>
+      <x:c r="H47" s="41" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I47" s="41" t="str">
+        <x:v>pytest tests/test_release_readiness.py</x:v>
+      </x:c>
+      <x:c r="J47" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K47" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L47" s="41" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M47" s="41" t="str">
+        <x:v>3 release-readiness tests passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="60" customHeight="1">
+      <x:c r="A48" s="41" t="str">
+        <x:v>TC-P01-025</x:v>
+      </x:c>
+      <x:c r="B48" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C48" s="41" t="str">
+        <x:v>Concurrent-session suspension</x:v>
+      </x:c>
+      <x:c r="D48" s="41" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E48" s="41" t="str">
+        <x:v>Two active requestor sessions and administrator</x:v>
+      </x:c>
+      <x:c r="F48" s="41" t="str">
+        <x:v>Suspend requestor while both sessions are active</x:v>
+      </x:c>
+      <x:c r="G48" s="41" t="str">
+        <x:v>Both sessions immediately return 401 and account can be safely restored</x:v>
+      </x:c>
+      <x:c r="H48" s="41" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I48" s="41" t="str">
+        <x:v>pytest test_suspension_revokes_all_concurrent_sessions</x:v>
+      </x:c>
+      <x:c r="J48" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K48" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L48" s="41" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M48" s="41" t="str">
+        <x:v>Isolated database; test state restored</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="60" customHeight="1">
+      <x:c r="A49" s="41" t="str">
+        <x:v>TC-P01-026</x:v>
+      </x:c>
+      <x:c r="B49" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C49" s="41" t="str">
+        <x:v>Large session cleanup batch</x:v>
+      </x:c>
+      <x:c r="D49" s="41" t="str">
+        <x:v>Maintenance</x:v>
+      </x:c>
+      <x:c r="E49" s="41" t="str">
+        <x:v>2,005 expired sessions and one active session</x:v>
+      </x:c>
+      <x:c r="F49" s="41" t="str">
+        <x:v>Clean with batch size 500</x:v>
+      </x:c>
+      <x:c r="G49" s="41" t="str">
+        <x:v>All 2,005 expired sessions are deleted across batches and active session remains</x:v>
+      </x:c>
+      <x:c r="H49" s="41" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I49" s="41" t="str">
+        <x:v>pytest test_cleanup_batches_thousands_without_removing_active_sessions</x:v>
+      </x:c>
+      <x:c r="J49" s="41" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K49" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L49" s="41" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M49" s="41" t="str">
+        <x:v>27-test suite; cleanup data removed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="60" customHeight="1">
+      <x:c r="A50" s="41" t="str">
+        <x:v>TC-P01-027</x:v>
+      </x:c>
+      <x:c r="B50" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C50" s="41" t="str">
+        <x:v>PostgreSQL backup and restore</x:v>
+      </x:c>
+      <x:c r="D50" s="41" t="str">
+        <x:v>Recovery</x:v>
+      </x:c>
+      <x:c r="E50" s="41" t="str">
+        <x:v>Migrated isolated database</x:v>
+      </x:c>
+      <x:c r="F50" s="41" t="str">
+        <x:v>pg_dump custom format; restore to fresh database; compare revision and table counts</x:v>
+      </x:c>
+      <x:c r="G50" s="41" t="str">
+        <x:v>Revision 20260826_0004 and sampled counts match exactly</x:v>
+      </x:c>
+      <x:c r="H50" s="41" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I50" s="41" t="str">
+        <x:v>pg_dump / pg_restore payment_module_test</x:v>
+      </x:c>
+      <x:c r="J50" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K50" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L50" s="41" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M50" s="41" t="str">
+        <x:v>Restore DB and dump removed after comparison</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="60" customHeight="1">
+      <x:c r="A51" s="41" t="str">
+        <x:v>TC-P01-028</x:v>
+      </x:c>
+      <x:c r="B51" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C51" s="41" t="str">
+        <x:v>Session continuity after API restart</x:v>
+      </x:c>
+      <x:c r="D51" s="41" t="str">
+        <x:v>Recovery</x:v>
+      </x:c>
+      <x:c r="E51" s="41" t="str">
+        <x:v>Disposable API container and authenticated test session</x:v>
+      </x:c>
+      <x:c r="F51" s="41" t="str">
+        <x:v>Restart API container; reuse session cookie</x:v>
+      </x:c>
+      <x:c r="G51" s="41" t="str">
+        <x:v>Session remains valid and returns 200 after restart</x:v>
+      </x:c>
+      <x:c r="H51" s="41" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I51" s="41" t="str">
+        <x:v>Disposable Docker API on port 8003</x:v>
+      </x:c>
+      <x:c r="J51" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K51" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L51" s="41" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M51" s="41" t="str">
+        <x:v>Required rebuilding stale local image; disposable resources removed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="60" customHeight="1">
+      <x:c r="A52" s="41" t="str">
+        <x:v>TC-P01-029</x:v>
+      </x:c>
+      <x:c r="B52" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C52" s="41" t="str">
+        <x:v>Python static security scan</x:v>
+      </x:c>
+      <x:c r="D52" s="41" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E52" s="41" t="str">
+        <x:v>Current API source</x:v>
+      </x:c>
+      <x:c r="F52" s="41" t="str">
+        <x:v>Run Bandit recursively excluding tests</x:v>
+      </x:c>
+      <x:c r="G52" s="41" t="str">
+        <x:v>No low, medium or high findings</x:v>
+      </x:c>
+      <x:c r="H52" s="41" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I52" s="41" t="str">
+        <x:v>bandit -r api -x tests</x:v>
+      </x:c>
+      <x:c r="J52" s="41" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K52" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L52" s="41" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M52" s="41" t="str">
+        <x:v>1,269 LOC scanned; zero findings</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="60" customHeight="1">
+      <x:c r="A53" s="41" t="str">
+        <x:v>TC-P01-030</x:v>
+      </x:c>
+      <x:c r="B53" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C53" s="41" t="str">
+        <x:v>Python dependency vulnerability audit</x:v>
+      </x:c>
+      <x:c r="D53" s="41" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E53" s="41" t="str">
+        <x:v>Installed runtime and test environment</x:v>
+      </x:c>
+      <x:c r="F53" s="41" t="str">
+        <x:v>Audit installed packages against current vulnerability data</x:v>
+      </x:c>
+      <x:c r="G53" s="41" t="str">
+        <x:v>No known vulnerable runtime dependencies</x:v>
+      </x:c>
+      <x:c r="H53" s="41" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I53" s="41" t="str">
+        <x:v>pip-audit --local --skip-editable</x:v>
+      </x:c>
+      <x:c r="J53" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K53" s="41" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="L53" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M53" s="41" t="str">
+        <x:v>Runtime findings include python-multipart 0.0.20 and Starlette 0.47.3; dev tooling also reported</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="60" customHeight="1">
+      <x:c r="A54" s="41" t="str">
+        <x:v>TC-P01-031</x:v>
+      </x:c>
+      <x:c r="B54" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C54" s="41" t="str">
+        <x:v>Frontend dependency vulnerability audit</x:v>
+      </x:c>
+      <x:c r="D54" s="41" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E54" s="41" t="str">
+        <x:v>Current pnpm lockfile</x:v>
+      </x:c>
+      <x:c r="F54" s="41" t="str">
+        <x:v>Run pnpm audit</x:v>
+      </x:c>
+      <x:c r="G54" s="41" t="str">
+        <x:v>No high or moderate vulnerabilities</x:v>
+      </x:c>
+      <x:c r="H54" s="41" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I54" s="41" t="str">
+        <x:v>pnpm audit</x:v>
+      </x:c>
+      <x:c r="J54" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K54" s="41" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="L54" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M54" s="41" t="str">
+        <x:v>9 advisories: 5 high and 4 moderate; includes xlsx, Vite, nanoid and postcss</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="60" customHeight="1">
+      <x:c r="A55" s="41" t="str">
+        <x:v>TC-P01-032</x:v>
+      </x:c>
+      <x:c r="B55" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C55" s="41" t="str">
+        <x:v>Integrated frontend production build</x:v>
+      </x:c>
+      <x:c r="D55" s="41" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="E55" s="41" t="str">
+        <x:v>Bundled Node runtime and installed dependencies</x:v>
+      </x:c>
+      <x:c r="F55" s="41" t="str">
+        <x:v>Run TypeScript and Vite production build</x:v>
+      </x:c>
+      <x:c r="G55" s="41" t="str">
+        <x:v>Build completes and emits HTML, CSS, application and XLSX chunks</x:v>
+      </x:c>
+      <x:c r="H55" s="41" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I55" s="41" t="str">
+        <x:v>pnpm run build</x:v>
+      </x:c>
+      <x:c r="J55" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K55" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L55" s="41" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M55" s="41" t="str">
+        <x:v>Vite build completed 2026-08-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="60" customHeight="1">
+      <x:c r="A56" s="41" t="str">
+        <x:v>TC-P01-033</x:v>
+      </x:c>
+      <x:c r="B56" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C56" s="41" t="str">
+        <x:v>Frontend/API proxy smoke test</x:v>
+      </x:c>
+      <x:c r="D56" s="41" t="str">
+        <x:v>Integration</x:v>
+      </x:c>
+      <x:c r="E56" s="41" t="str">
+        <x:v>Integrated frontend on 5176; API on 8002</x:v>
+      </x:c>
+      <x:c r="F56" s="41" t="str">
+        <x:v>Load root; login and logout through Vite proxy</x:v>
+      </x:c>
+      <x:c r="G56" s="41" t="str">
+        <x:v>Root returns 200; proxy login succeeds; logout returns 204</x:v>
+      </x:c>
+      <x:c r="H56" s="41" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I56" s="41" t="str">
+        <x:v>HTTP smoke test against 127.0.0.1:5176</x:v>
+      </x:c>
+      <x:c r="J56" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K56" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L56" s="41" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M56" s="41" t="str">
+        <x:v>Frontend-only port 5175 was not used</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="60" customHeight="1">
+      <x:c r="A57" s="41" t="str">
+        <x:v>TC-P01-034</x:v>
+      </x:c>
+      <x:c r="B57" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C57" s="41" t="str">
+        <x:v>Responsive and accessibility walkthrough</x:v>
+      </x:c>
+      <x:c r="D57" s="41" t="str">
+        <x:v>UI</x:v>
+      </x:c>
+      <x:c r="E57" s="41" t="str">
+        <x:v>Interactive browser automation available</x:v>
+      </x:c>
+      <x:c r="F57" s="41" t="str">
+        <x:v>Test admin pages, modals, keyboard flow, labels and narrow layouts</x:v>
+      </x:c>
+      <x:c r="G57" s="41" t="str">
+        <x:v>No alignment, focus, naming or overflow defects</x:v>
+      </x:c>
+      <x:c r="H57" s="41" t="str">
+        <x:v>Manual</x:v>
+      </x:c>
+      <x:c r="I57" s="41" t="str">
+        <x:v>In-app browser walkthrough</x:v>
+      </x:c>
+      <x:c r="J57" s="41" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K57" s="41" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="L57" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M57" s="41" t="str">
+        <x:v>Browser automation runtime failed to load; requires rerun in an interactive browser</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="60" customHeight="1">
+      <x:c r="A58" s="41" t="str">
+        <x:v>TC-P01-035</x:v>
+      </x:c>
+      <x:c r="B58" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C58" s="41" t="str">
+        <x:v>Cross-browser compatibility</x:v>
+      </x:c>
+      <x:c r="D58" s="41" t="str">
+        <x:v>UI</x:v>
+      </x:c>
+      <x:c r="E58" s="41" t="str">
+        <x:v>Chrome, Firefox and Safari environments</x:v>
+      </x:c>
+      <x:c r="F58" s="41" t="str">
+        <x:v>Run authentication and administration smoke paths in each browser</x:v>
+      </x:c>
+      <x:c r="G58" s="41" t="str">
+        <x:v>Supported browsers render and behave consistently</x:v>
+      </x:c>
+      <x:c r="H58" s="41" t="str">
+        <x:v>Manual</x:v>
+      </x:c>
+      <x:c r="I58" s="41" t="str">
+        <x:v>External browser matrix</x:v>
+      </x:c>
+      <x:c r="J58" s="41" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K58" s="41" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="L58" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M58" s="41" t="str">
+        <x:v>Only local Chromium surface is available; Firefox and Safari were not executed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="60" customHeight="1">
+      <x:c r="A59" s="41" t="str">
+        <x:v>TC-P01-036</x:v>
+      </x:c>
+      <x:c r="B59" s="41" t="str">
+        <x:v>P01</x:v>
+      </x:c>
+      <x:c r="C59" s="41" t="str">
+        <x:v>Downloaded Excel workbook integrity</x:v>
+      </x:c>
+      <x:c r="D59" s="41" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="E59" s="41" t="str">
+        <x:v>Interactive browser download available</x:v>
+      </x:c>
+      <x:c r="F59" s="41" t="str">
+        <x:v>Export filtered department report; reopen workbook and validate sheets/filters</x:v>
+      </x:c>
+      <x:c r="G59" s="41" t="str">
+        <x:v>Valid XLSX contains Summary and Transactions sheets matching active filters</x:v>
+      </x:c>
+      <x:c r="H59" s="41" t="str">
+        <x:v>Manual</x:v>
+      </x:c>
+      <x:c r="I59" s="41" t="str">
+        <x:v>Dashboard &gt; Export Excel &gt; reopen workbook</x:v>
+      </x:c>
+      <x:c r="J59" s="41" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K59" s="41" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="L59" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M59" s="41" t="str">
+        <x:v>Implementation and build pass, but an actual browser download was not captured</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4791,7 +5414,7 @@
     <x:cfRule type="containsText" dxfId="26" priority="6" operator="containsText" text="Not Run"/>
     <x:cfRule type="containsText" dxfId="27" priority="7" operator="containsText" text="Pending"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="6">
+  <x:dataValidations count="9">
     <x:dataValidation type="list" sqref="J4:J300">
       <x:formula1>"Critical,High,Medium,Low"</x:formula1>
     </x:dataValidation>
@@ -4810,10 +5433,19 @@
     <x:dataValidation type="list" sqref="L24:L45">
       <x:formula1>"Yes,No"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="J46:J59">
+      <x:formula1>"Critical,High,Medium,Low"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="K46:K59">
+      <x:formula1>"Not Run,Passed,Failed,Blocked,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="L46:L59">
+      <x:formula1>"Yes,No"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b4cba769e1a4cda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb78921d86b624362"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6377,10 +7009,10 @@
         <x:v>a796a43</x:v>
       </x:c>
       <x:c r="F45" s="41" t="str">
-        <x:v>Executed</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G45" s="41" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H45" s="41" t="str">
         <x:v>XLSX export implementation and build passed</x:v>
@@ -6390,10 +7022,518 @@
       </x:c>
       <x:c r="J45" s="41"/>
       <x:c r="K45" s="41" t="str">
-        <x:v>No</x:v>
+        <x:v>Required</x:v>
       </x:c>
       <x:c r="L45" s="41" t="str">
         <x:v>Evidence recorded in docs/phase-01-plan.md and PROJECT_MANIFEST.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="60" customHeight="1">
+      <x:c r="A46" s="41" t="str">
+        <x:v>RUN-20260827-001</x:v>
+      </x:c>
+      <x:c r="B46" s="41" t="str">
+        <x:v>TC-P01-023</x:v>
+      </x:c>
+      <x:c r="C46" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D46" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E46" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F46" s="41" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G46" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H46" s="41" t="str">
+        <x:v>Isolated PostgreSQL 16 validation 2026-08-27</x:v>
+      </x:c>
+      <x:c r="I46" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J46" s="41"/>
+      <x:c r="K46" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="L46" s="41" t="str">
+        <x:v>Isolated PostgreSQL 16 validation 2026-08-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="60" customHeight="1">
+      <x:c r="A47" s="41" t="str">
+        <x:v>RUN-20260827-002</x:v>
+      </x:c>
+      <x:c r="B47" s="41" t="str">
+        <x:v>TC-P01-024</x:v>
+      </x:c>
+      <x:c r="C47" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D47" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E47" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F47" s="41" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G47" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H47" s="41" t="str">
+        <x:v>3 release-readiness tests passed</x:v>
+      </x:c>
+      <x:c r="I47" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J47" s="41"/>
+      <x:c r="K47" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="L47" s="41" t="str">
+        <x:v>3 release-readiness tests passed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="60" customHeight="1">
+      <x:c r="A48" s="41" t="str">
+        <x:v>RUN-20260827-003</x:v>
+      </x:c>
+      <x:c r="B48" s="41" t="str">
+        <x:v>TC-P01-025</x:v>
+      </x:c>
+      <x:c r="C48" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D48" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E48" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F48" s="41" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G48" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H48" s="41" t="str">
+        <x:v>Isolated database; test state restored</x:v>
+      </x:c>
+      <x:c r="I48" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J48" s="41"/>
+      <x:c r="K48" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="L48" s="41" t="str">
+        <x:v>Isolated database; test state restored</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="60" customHeight="1">
+      <x:c r="A49" s="41" t="str">
+        <x:v>RUN-20260827-004</x:v>
+      </x:c>
+      <x:c r="B49" s="41" t="str">
+        <x:v>TC-P01-026</x:v>
+      </x:c>
+      <x:c r="C49" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D49" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E49" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F49" s="41" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G49" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H49" s="41" t="str">
+        <x:v>27-test suite; cleanup data removed</x:v>
+      </x:c>
+      <x:c r="I49" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J49" s="41"/>
+      <x:c r="K49" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="L49" s="41" t="str">
+        <x:v>27-test suite; cleanup data removed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="60" customHeight="1">
+      <x:c r="A50" s="41" t="str">
+        <x:v>RUN-20260827-005</x:v>
+      </x:c>
+      <x:c r="B50" s="41" t="str">
+        <x:v>TC-P01-027</x:v>
+      </x:c>
+      <x:c r="C50" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D50" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E50" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F50" s="41" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G50" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H50" s="41" t="str">
+        <x:v>Restore DB and dump removed after comparison</x:v>
+      </x:c>
+      <x:c r="I50" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J50" s="41"/>
+      <x:c r="K50" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="L50" s="41" t="str">
+        <x:v>Restore DB and dump removed after comparison</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="60" customHeight="1">
+      <x:c r="A51" s="41" t="str">
+        <x:v>RUN-20260827-006</x:v>
+      </x:c>
+      <x:c r="B51" s="41" t="str">
+        <x:v>TC-P01-028</x:v>
+      </x:c>
+      <x:c r="C51" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D51" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E51" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F51" s="41" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G51" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H51" s="41" t="str">
+        <x:v>Required rebuilding stale local image; disposable resources removed</x:v>
+      </x:c>
+      <x:c r="I51" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J51" s="41"/>
+      <x:c r="K51" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="L51" s="41" t="str">
+        <x:v>Required rebuilding stale local image; disposable resources removed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="60" customHeight="1">
+      <x:c r="A52" s="41" t="str">
+        <x:v>RUN-20260827-007</x:v>
+      </x:c>
+      <x:c r="B52" s="41" t="str">
+        <x:v>TC-P01-029</x:v>
+      </x:c>
+      <x:c r="C52" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D52" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E52" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F52" s="41" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G52" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H52" s="41" t="str">
+        <x:v>1,269 LOC scanned; zero findings</x:v>
+      </x:c>
+      <x:c r="I52" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J52" s="41"/>
+      <x:c r="K52" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="L52" s="41" t="str">
+        <x:v>1,269 LOC scanned; zero findings</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="60" customHeight="1">
+      <x:c r="A53" s="41" t="str">
+        <x:v>RUN-20260827-008</x:v>
+      </x:c>
+      <x:c r="B53" s="41" t="str">
+        <x:v>TC-P01-030</x:v>
+      </x:c>
+      <x:c r="C53" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D53" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E53" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F53" s="41" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G53" s="41" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="H53" s="41" t="str">
+        <x:v>Runtime findings include python-multipart 0.0.20 and Starlette 0.47.3; dev tooling also reported</x:v>
+      </x:c>
+      <x:c r="I53" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J53" s="41" t="str">
+        <x:v>Dependency remediation required</x:v>
+      </x:c>
+      <x:c r="K53" s="41" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="L53" s="41" t="str">
+        <x:v>Runtime findings include python-multipart 0.0.20 and Starlette 0.47.3; dev tooling also reported</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="60" customHeight="1">
+      <x:c r="A54" s="41" t="str">
+        <x:v>RUN-20260827-009</x:v>
+      </x:c>
+      <x:c r="B54" s="41" t="str">
+        <x:v>TC-P01-031</x:v>
+      </x:c>
+      <x:c r="C54" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D54" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E54" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F54" s="41" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G54" s="41" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="H54" s="41" t="str">
+        <x:v>9 advisories: 5 high and 4 moderate; includes xlsx, Vite, nanoid and postcss</x:v>
+      </x:c>
+      <x:c r="I54" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J54" s="41" t="str">
+        <x:v>Dependency remediation required</x:v>
+      </x:c>
+      <x:c r="K54" s="41" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="L54" s="41" t="str">
+        <x:v>9 advisories: 5 high and 4 moderate; includes xlsx, Vite, nanoid and postcss</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="60" customHeight="1">
+      <x:c r="A55" s="41" t="str">
+        <x:v>RUN-20260827-010</x:v>
+      </x:c>
+      <x:c r="B55" s="41" t="str">
+        <x:v>TC-P01-032</x:v>
+      </x:c>
+      <x:c r="C55" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D55" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E55" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F55" s="41" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G55" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H55" s="41" t="str">
+        <x:v>Vite build completed 2026-08-27</x:v>
+      </x:c>
+      <x:c r="I55" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J55" s="41"/>
+      <x:c r="K55" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="L55" s="41" t="str">
+        <x:v>Vite build completed 2026-08-27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="60" customHeight="1">
+      <x:c r="A56" s="41" t="str">
+        <x:v>RUN-20260827-011</x:v>
+      </x:c>
+      <x:c r="B56" s="41" t="str">
+        <x:v>TC-P01-033</x:v>
+      </x:c>
+      <x:c r="C56" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D56" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E56" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F56" s="41" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G56" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H56" s="41" t="str">
+        <x:v>Frontend-only port 5175 was not used</x:v>
+      </x:c>
+      <x:c r="I56" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J56" s="41"/>
+      <x:c r="K56" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="L56" s="41" t="str">
+        <x:v>Frontend-only port 5175 was not used</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="60" customHeight="1">
+      <x:c r="A57" s="41" t="str">
+        <x:v>RUN-20260827-012</x:v>
+      </x:c>
+      <x:c r="B57" s="41" t="str">
+        <x:v>TC-P01-034</x:v>
+      </x:c>
+      <x:c r="C57" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D57" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E57" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F57" s="41" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="G57" s="41" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="H57" s="41" t="str">
+        <x:v>Browser automation runtime failed to load; requires rerun in an interactive browser</x:v>
+      </x:c>
+      <x:c r="I57" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J57" s="41"/>
+      <x:c r="K57" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="L57" s="41" t="str">
+        <x:v>Browser automation runtime failed to load; requires rerun in an interactive browser</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="60" customHeight="1">
+      <x:c r="A58" s="41" t="str">
+        <x:v>RUN-20260827-013</x:v>
+      </x:c>
+      <x:c r="B58" s="41" t="str">
+        <x:v>TC-P01-035</x:v>
+      </x:c>
+      <x:c r="C58" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D58" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E58" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F58" s="41" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="G58" s="41" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="H58" s="41" t="str">
+        <x:v>Only local Chromium surface is available; Firefox and Safari were not executed</x:v>
+      </x:c>
+      <x:c r="I58" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J58" s="41"/>
+      <x:c r="K58" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="L58" s="41" t="str">
+        <x:v>Only local Chromium surface is available; Firefox and Safari were not executed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="60" customHeight="1">
+      <x:c r="A59" s="41" t="str">
+        <x:v>RUN-20260827-014</x:v>
+      </x:c>
+      <x:c r="B59" s="41" t="str">
+        <x:v>TC-P01-036</x:v>
+      </x:c>
+      <x:c r="C59" s="42" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="D59" s="41" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7</x:v>
+      </x:c>
+      <x:c r="E59" s="41" t="str">
+        <x:v>working tree after acb887f</x:v>
+      </x:c>
+      <x:c r="F59" s="41" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="G59" s="41" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="H59" s="41" t="str">
+        <x:v>Implementation and build pass, but an actual browser download was not captured</x:v>
+      </x:c>
+      <x:c r="I59" s="41" t="str">
+        <x:v>Codex local release-readiness audit</x:v>
+      </x:c>
+      <x:c r="J59" s="41"/>
+      <x:c r="K59" s="41" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="L59" s="41" t="str">
+        <x:v>Implementation and build pass, but an actual browser download was not captured</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6410,7 +7550,7 @@
     <x:cfRule type="containsText" dxfId="33" priority="6" operator="containsText" text="Not Run"/>
     <x:cfRule type="containsText" dxfId="34" priority="7" operator="containsText" text="Pending"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="6">
+  <x:dataValidations count="9">
     <x:dataValidation type="list" sqref="F4:F500">
       <x:formula1>"Pending,Executed,Blocked"</x:formula1>
     </x:dataValidation>
@@ -6429,10 +7569,19 @@
     <x:dataValidation type="list" sqref="K24:K45">
       <x:formula1>"No,Required,Completed"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="F46:F59">
+      <x:formula1>"Not Run,Executed,Blocked"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G46:G59">
+      <x:formula1>"Not Run,Passed,Failed,Blocked,N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="K46:K59">
+      <x:formula1>"No,Required,Completed"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb838d04c169454a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0eb1ca13ff14ca8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6899,10 +8048,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="G16" s="41" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H16" s="41" t="str">
-        <x:v>Standalone build/routes and XLSX export passed</x:v>
+        <x:v>Standalone build passed; actual Excel download and cross-browser UI validation remain</x:v>
       </x:c>
       <x:c r="I16" s="42" t="n">
         <x:v>46260</x:v>
@@ -6931,10 +8080,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="G17" s="41" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H17" s="41" t="str">
-        <x:v>23 tests; 90.46% coverage; commit a796a43</x:v>
+        <x:v>Functional gates pass; Python and frontend dependency audits contain release blockers</x:v>
       </x:c>
       <x:c r="I17" s="42" t="n">
         <x:v>46260</x:v>
@@ -6970,7 +8119,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a3ea9e6bb304349"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66c4894fdcdb4473"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7220,6 +8369,6 @@
     <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea4621a0ede54191"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46c6403ba8fb44be"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: validate phase 01 release
</commit_message>
<xml_diff>
--- a/Back End/outputs/development-test-register/APS-Development-and-Test-Register-Phase-01.xlsx
+++ b/Back End/outputs/development-test-register/APS-Development-and-Test-Register-Phase-01.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R999a5b56e8494e5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Register" sheetId="2" r:id="R144d7cc2825e4c1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Log" sheetId="3" r:id="R2acb00e4f0374739"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="4" r:id="R4ac50ca2de2e48a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Executions" sheetId="5" r:id="Rc7d14a82ddf249d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="6" r:id="R794fe10da0c245ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="7" r:id="Ra2dbdc5c6fff40d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R25405fd34e9c426a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Register" sheetId="2" r:id="R8052b8ca785043b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Log" sheetId="3" r:id="R85bc16dc97d64635"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="4" r:id="Rdb2e81b7ee864faf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Executions" sheetId="5" r:id="R392bb44962464c05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="6" r:id="Rfb5bf3af51e64c4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="7" r:id="Rd3efc6dc80d5402f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -179,7 +179,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="57">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -323,6 +323,7 @@
     <x:xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -930,7 +931,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R29995a806f344281"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdf68ca5f452149de"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1295,7 +1296,7 @@
         <x:v>Functional suite</x:v>
       </x:c>
       <x:c r="E5" s="46" t="str">
-        <x:v>27 passed</x:v>
+        <x:v>28 passed</x:v>
       </x:c>
       <x:c r="F5" s="51" t="str">
         <x:v>Passed</x:v>
@@ -1303,8 +1304,8 @@
       <x:c r="G5" s="22" t="str">
         <x:v>90.59% coverage</x:v>
       </x:c>
-      <x:c r="H5" s="22" t="str">
-        <x:v>2026-08-27</x:v>
+      <x:c r="H5" s="37" t="n">
+        <x:v>46262</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="60" hidden="0" customHeight="1">
@@ -1327,8 +1328,8 @@
       <x:c r="G6" s="23" t="str">
         <x:v>Revision and sampled counts matched</x:v>
       </x:c>
-      <x:c r="H6" s="23" t="str">
-        <x:v>2026-08-27</x:v>
+      <x:c r="H6" s="38" t="n">
+        <x:v>46262</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="84" hidden="0" customHeight="1">
@@ -1336,8 +1337,7 @@
         <x:v>Passed tests</x:v>
       </x:c>
       <x:c r="B7" s="32" t="n">
-        <x:f>COUNTIF('Test Executions'!$G$4:$G$60,"Passed")</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
         <x:v>Session resilience</x:v>
@@ -1351,8 +1351,8 @@
       <x:c r="G7" s="23" t="str">
         <x:v>Distinct sessions; restart continuity</x:v>
       </x:c>
-      <x:c r="H7" s="23" t="str">
-        <x:v>2026-08-27</x:v>
+      <x:c r="H7" s="38" t="n">
+        <x:v>46262</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="72" hidden="0" customHeight="1">
@@ -1360,8 +1360,7 @@
         <x:v>Failed tests</x:v>
       </x:c>
       <x:c r="B8" s="32" t="n">
-        <x:f>COUNTIF('Test Executions'!$G$4:$G$60,"Failed")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
         <x:v>Python dependencies</x:v>
@@ -1370,22 +1369,21 @@
         <x:v>pip-audit</x:v>
       </x:c>
       <x:c r="F8" s="54" t="str">
-        <x:v>Failed</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G8" s="23" t="str">
-        <x:v>Runtime vulnerabilities require remediation</x:v>
-      </x:c>
-      <x:c r="H8" s="23" t="str">
-        <x:v>2026-08-27</x:v>
+        <x:v>No known vulnerabilities</x:v>
+      </x:c>
+      <x:c r="H8" s="38" t="n">
+        <x:v>46262</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="60" hidden="0" customHeight="1">
       <x:c r="A9" s="24" t="str">
-        <x:v>Not-run tests</x:v>
+        <x:v>Blocked tests</x:v>
       </x:c>
       <x:c r="B9" s="33" t="n">
-        <x:f>COUNTIF('Test Executions'!$G$4:$G$60,"Not Run")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
         <x:v>Frontend dependencies</x:v>
@@ -1394,30 +1392,32 @@
         <x:v>pnpm audit</x:v>
       </x:c>
       <x:c r="F9" s="54" t="str">
-        <x:v>Failed</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G9" s="23" t="str">
-        <x:v>5 high and 4 moderate advisories</x:v>
-      </x:c>
-      <x:c r="H9" s="23" t="str">
-        <x:v>2026-08-27</x:v>
+        <x:v>No known vulnerabilities</x:v>
+      </x:c>
+      <x:c r="H9" s="38" t="n">
+        <x:v>46262</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="84" hidden="0" customHeight="1">
+      <x:c r="A10"/>
+      <x:c r="B10"/>
       <x:c r="D10" s="24" t="str">
         <x:v>Browser matrix</x:v>
       </x:c>
       <x:c r="E10" s="48" t="str">
-        <x:v>Interactive/cross-browser</x:v>
+        <x:v>Chrome + in-app</x:v>
       </x:c>
       <x:c r="F10" s="56" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Accepted limitation</x:v>
       </x:c>
       <x:c r="G10" s="24" t="str">
-        <x:v>Browser runtime and external browsers required</x:v>
-      </x:c>
-      <x:c r="H10" s="24" t="str">
-        <x:v>2026-08-27</x:v>
+        <x:v>Firefox/Safari required before production promotion</x:v>
+      </x:c>
+      <x:c r="H10" s="39" t="n">
+        <x:v>46262</x:v>
       </x:c>
     </x:row>
     <x:row r="11"/>
@@ -1434,8 +1434,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="E13" t="n">
-        <x:f>B7</x:f>
-        <x:v>50</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -1443,17 +1442,15 @@
         <x:v>Failed</x:v>
       </x:c>
       <x:c r="E14" t="n">
-        <x:f>B8</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="D15" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="E15" t="n">
-        <x:f>B9</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16"/>
@@ -1477,7 +1474,7 @@
         <x:v>Commit</x:v>
       </x:c>
       <x:c r="G18" s="22" t="str">
-        <x:v>a796a43</x:v>
+        <x:v>44e876e</x:v>
       </x:c>
       <x:c r="H18" s="22"/>
     </x:row>
@@ -1536,8 +1533,8 @@
       <x:c r="F22" s="24" t="str">
         <x:v>Updated</x:v>
       </x:c>
-      <x:c r="G22" s="24" t="str">
-        <x:v>2026-08-27</x:v>
+      <x:c r="G22" s="39" t="n">
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="H22" s="24"/>
     </x:row>
@@ -1558,7 +1555,7 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="Pending"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19d1701f29b14178"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f8c3f5630a94a57"/>
 </x:worksheet>
 </file>
 
@@ -1665,13 +1662,13 @@
         <x:v>docs/phase-01-plan.md</x:v>
       </x:c>
       <x:c r="G5" s="38" t="n">
-        <x:v>46260</x:v>
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="H5" s="23" t="str">
         <x:v>Backend Team</x:v>
       </x:c>
       <x:c r="I5" s="23" t="str">
-        <x:v>27 tests passed; 90.59% coverage. Release blocked by dependency vulnerabilities and interactive browser validation gaps.</x:v>
+        <x:v>28 tests passed; 90.59% coverage; clean Python/frontend audits; Chrome/in-app UI and XLSX integrity passed. Firefox, Safari, penetration, and production proxy/HTTPS checks are accepted production-promotion limitations.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="120" hidden="0" customHeight="1">
@@ -1911,7 +1908,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb395cd659c0c43be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd118844ae4a24bdb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2917,19 +2914,19 @@
         <x:v>codex/backend-integration</x:v>
       </x:c>
       <x:c r="H28" s="41" t="str">
-        <x:v>a796a43</x:v>
+        <x:v>44e876e</x:v>
       </x:c>
       <x:c r="I28" s="41" t="str">
-        <x:v>Export Excel</x:v>
+        <x:v>Export Excel + verified XLSX</x:v>
       </x:c>
       <x:c r="J28" s="41" t="str">
         <x:v>Frontend Team</x:v>
       </x:c>
       <x:c r="K28" s="42" t="n">
-        <x:v>46260</x:v>
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="L28" s="41" t="str">
-        <x:v>Department report produces an XLSX workbook</x:v>
+        <x:v>Filtered Finance report reopened with correct sheets, rows, and total</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="54" customHeight="1">
@@ -2955,19 +2952,19 @@
         <x:v>codex/backend-integration</x:v>
       </x:c>
       <x:c r="H29" s="41" t="str">
-        <x:v>a796a43</x:v>
+        <x:v>44e876e</x:v>
       </x:c>
       <x:c r="I29" s="41" t="str">
-        <x:v>23 tests / 90.46% / release archive</x:v>
+        <x:v>28 tests / 90.59% / clean audits / release archive</x:v>
       </x:c>
       <x:c r="J29" s="41" t="str">
         <x:v>Paolo Ylag</x:v>
       </x:c>
       <x:c r="K29" s="42" t="n">
-        <x:v>46260</x:v>
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="L29" s="41" t="str">
-        <x:v>Local release gates and production refusal passed</x:v>
+        <x:v>Local release gates passed; external production-promotion checks recorded</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
@@ -3029,7 +3026,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3c87407b9124436"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d96d21a830a42b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4817,13 +4814,13 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="K45" s="41" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="L45" s="41" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M45" s="41" t="str">
-        <x:v>Implementation/build passed; actual downloaded workbook validation remains blocked</x:v>
+        <x:v>Finance-filtered XLSX reopened: Summary + Transactions, 2 rows, PHP 113,850</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="60" customHeight="1">
@@ -5145,13 +5142,13 @@
         <x:v>Critical</x:v>
       </x:c>
       <x:c r="K53" s="41" t="str">
-        <x:v>Failed</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="L53" s="41" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M53" s="41" t="str">
-        <x:v>Runtime findings include python-multipart 0.0.20 and Starlette 0.47.3; dev tooling also reported</x:v>
+        <x:v>pip-audit found no known vulnerabilities after runtime dependency remediation</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="60" customHeight="1">
@@ -5186,13 +5183,13 @@
         <x:v>Critical</x:v>
       </x:c>
       <x:c r="K54" s="41" t="str">
-        <x:v>Failed</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="L54" s="41" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M54" s="41" t="str">
-        <x:v>9 advisories: 5 high and 4 moderate; includes xlsx, Vite, nanoid and postcss</x:v>
+        <x:v>pnpm audit found no known vulnerabilities; SheetJS 0.20.3 vendored from official distribution</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="60" customHeight="1">
@@ -5309,13 +5306,13 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="K57" s="41" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="L57" s="41" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M57" s="41" t="str">
-        <x:v>Browser automation runtime failed to load; requires rerun in an interactive browser</x:v>
+        <x:v>Desktop/mobile administration walkthrough found no overflow, unnamed buttons, or unlabeled controls</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="60" customHeight="1">
@@ -5356,7 +5353,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="M58" s="41" t="str">
-        <x:v>Only local Chromium surface is available; Firefox and Safari were not executed</x:v>
+        <x:v>Chrome and in-app Chromium passed; Firefox and Safari unavailable on Windows host</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="60" customHeight="1">
@@ -5391,13 +5388,13 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="K59" s="41" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="L59" s="41" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M59" s="41" t="str">
-        <x:v>Implementation and build pass, but an actual browser download was not captured</x:v>
+        <x:v>Downloaded workbook sheets, filters, totals, and formula-error scan passed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5445,7 +5442,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb78921d86b624362"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R359d9b89381a4fcc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7535,6 +7532,188 @@
       <x:c r="L59" s="41" t="str">
         <x:v>Implementation and build pass, but an actual browser download was not captured</x:v>
       </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>RUN-20260828-001</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>TC-P01-022</x:v>
+      </x:c>
+      <x:c r="C60" s="57" t="n">
+        <x:v>46262</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7.3.6 / Chrome</x:v>
+      </x:c>
+      <x:c r="E60" t="str">
+        <x:v>44e876e</x:v>
+      </x:c>
+      <x:c r="F60" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>Finance filter downloaded a valid XLSX: Summary + Transactions, 2 rows, PHP 113,850</x:v>
+      </x:c>
+      <x:c r="I60" t="str">
+        <x:v>Codex final Phase 01 validation</x:v>
+      </x:c>
+      <x:c r="J60"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>RUN-20260828-002</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>TC-P01-030</x:v>
+      </x:c>
+      <x:c r="C61" s="57" t="n">
+        <x:v>46262</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7.3.6 / Chrome</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>44e876e</x:v>
+      </x:c>
+      <x:c r="F61" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>pip-audit: no known vulnerabilities after dependency remediation</x:v>
+      </x:c>
+      <x:c r="I61" t="str">
+        <x:v>Codex final Phase 01 validation</x:v>
+      </x:c>
+      <x:c r="J61"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="str">
+        <x:v>RUN-20260828-003</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>TC-P01-031</x:v>
+      </x:c>
+      <x:c r="C62" s="57" t="n">
+        <x:v>46262</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7.3.6 / Chrome</x:v>
+      </x:c>
+      <x:c r="E62" t="str">
+        <x:v>44e876e</x:v>
+      </x:c>
+      <x:c r="F62" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G62" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>pnpm audit: no known vulnerabilities; official SheetJS 0.20.3 package vendored</x:v>
+      </x:c>
+      <x:c r="I62" t="str">
+        <x:v>Codex final Phase 01 validation</x:v>
+      </x:c>
+      <x:c r="J62"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="str">
+        <x:v>RUN-20260828-004</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>TC-P01-034</x:v>
+      </x:c>
+      <x:c r="C63" s="57" t="n">
+        <x:v>46262</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7.3.6 / Chrome</x:v>
+      </x:c>
+      <x:c r="E63" t="str">
+        <x:v>44e876e</x:v>
+      </x:c>
+      <x:c r="F63" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G63" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H63" t="str">
+        <x:v>In-app browser desktop/mobile admin walkthrough passed naming, labels, modal containment, and overflow checks</x:v>
+      </x:c>
+      <x:c r="I63" t="str">
+        <x:v>Codex final Phase 01 validation</x:v>
+      </x:c>
+      <x:c r="J63"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
+        <x:v>RUN-20260828-005</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>TC-P01-035</x:v>
+      </x:c>
+      <x:c r="C64" s="57" t="n">
+        <x:v>46262</x:v>
+      </x:c>
+      <x:c r="D64" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7.3.6 / Chrome</x:v>
+      </x:c>
+      <x:c r="E64" t="str">
+        <x:v>44e876e</x:v>
+      </x:c>
+      <x:c r="F64" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G64" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="H64" t="str">
+        <x:v>Desktop Chrome and in-app Chromium passed; Firefox and Safari unavailable on this Windows host</x:v>
+      </x:c>
+      <x:c r="I64" t="str">
+        <x:v>Codex final Phase 01 validation</x:v>
+      </x:c>
+      <x:c r="J64" t="str">
+        <x:v>Accepted limitation; execute before production promotion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>RUN-20260828-006</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>TC-P01-036</x:v>
+      </x:c>
+      <x:c r="C65" s="57" t="n">
+        <x:v>46262</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>Windows / Docker Desktop / PostgreSQL 16 / Vite 7.3.6 / Chrome</x:v>
+      </x:c>
+      <x:c r="E65" t="str">
+        <x:v>44e876e</x:v>
+      </x:c>
+      <x:c r="F65" t="str">
+        <x:v>Executed</x:v>
+      </x:c>
+      <x:c r="G65" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="H65" t="str">
+        <x:v>Downloaded workbook reopened successfully; filters, totals, sheets, and formula-error scan passed</x:v>
+      </x:c>
+      <x:c r="I65" t="str">
+        <x:v>Codex final Phase 01 validation</x:v>
+      </x:c>
+      <x:c r="J65"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -7581,7 +7760,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0eb1ca13ff14ca8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6eeec06c02e74993"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8048,13 +8227,13 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="G16" s="41" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Accepted</x:v>
       </x:c>
       <x:c r="H16" s="41" t="str">
-        <x:v>Standalone build passed; actual Excel download and cross-browser UI validation remain</x:v>
+        <x:v>Standalone mock mode and real filtered Excel export passed</x:v>
       </x:c>
       <x:c r="I16" s="42" t="n">
-        <x:v>46260</x:v>
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="J16" s="41" t="str">
         <x:v>Paolo Ylag</x:v>
@@ -8080,13 +8259,13 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="G17" s="41" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Accepted</x:v>
       </x:c>
       <x:c r="H17" s="41" t="str">
-        <x:v>Functional gates pass; Python and frontend dependency audits contain release blockers</x:v>
+        <x:v>28 tests, 90.59% coverage, clean dependency audits, build, package, and local browser checks passed</x:v>
       </x:c>
       <x:c r="I17" s="42" t="n">
-        <x:v>46260</x:v>
+        <x:v>46262</x:v>
       </x:c>
       <x:c r="J17" s="41" t="str">
         <x:v>Paolo Ylag</x:v>
@@ -8119,7 +8298,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66c4894fdcdb4473"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f7c30519f9943bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8369,6 +8548,6 @@
     <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46c6403ba8fb44be"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32ac00333c3a4011"/>
 </x:worksheet>
 </file>
</xml_diff>